<commit_message>
Landowner presentations: D-132 (no boosters, cove LED rate, common BOQ refresh)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011zFSzvwKswJ2bde5abTBN3
</commit_message>
<xml_diff>
--- a/public/landowner-presentation/files/BOQ-77-76-Common-Works.xlsx
+++ b/public/landowner-presentation/files/BOQ-77-76-Common-Works.xlsx
@@ -7058,24 +7058,24 @@
       </c>
       <c r="B211" s="5" t="inlineStr">
         <is>
-          <t>Booster sets for floors 4–5, 1 working + 1 standby per block</t>
+          <t>Raised OHT staging 10 ft (3.05 m) to the tank base + floors 4–5 zone pipes upsized; no booster pumps (Plumbing Rev P1, D-132)</t>
         </is>
       </c>
       <c r="C211" s="5" t="inlineStr">
         <is>
-          <t>≈ 0.37 kW each, pressure vessel, controller · Grundfos / CRI (to quote)</t>
+          <t>Gravity supply to every floor: staging columns and ring beam by the structural engineer (≈ 22 t full tank); header 2″, down-takes 1¼″, branches 1″ on floors 4–5; 5th-floor low-pressure showers · Structural engineer / plumber</t>
         </is>
       </c>
       <c r="D211" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>sets</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F211" s="6" t="n">
-        <v>85000</v>
+        <v>75000</v>
       </c>
       <c r="G211" s="7">
         <f>D211*F211</f>
@@ -7771,16 +7771,12 @@
       </c>
       <c r="B234" s="5" t="inlineStr">
         <is>
-          <t>Feeders 4C/3C × 2.5–6 sq mm Cu armoured (lift, pumps, boosters, common DBs, gates, watchman, CCTV, DG)</t>
-        </is>
-      </c>
-      <c r="C234" s="5" t="inlineStr">
-        <is>
-          <t>Polycab</t>
-        </is>
-      </c>
+          <t>Feeders 4C/3C × 2.5–6 sq mm Cu armoured (lift, pumps, common DBs, gates, watchman, CCTV, DG)</t>
+        </is>
+      </c>
+      <c r="C234" s="5" t="n"/>
       <c r="D234" s="6" t="n">
-        <v>330</v>
+        <v>248</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>

</xml_diff>